<commit_message>
chore: run 2026-05-18 09:53 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_18_05_2026.xlsx
+++ b/logs/Consolidado_18_05_2026.xlsx
@@ -679,7 +679,7 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>11</v>
@@ -736,7 +736,7 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>15</v>
@@ -7976,7 +7976,11 @@
           <t>Out of Stock</t>
         </is>
       </c>
-      <c r="G18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>5976179</t>
+        </is>
+      </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
           <t>25%</t>
@@ -10593,7 +10597,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>6935360</t>
+        </is>
+      </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
           <t>20%</t>

</xml_diff>